<commit_message>
sheet tweaks and edit lunch
</commit_message>
<xml_diff>
--- a/escala_triagem_ajustada.xlsx
+++ b/escala_triagem_ajustada.xlsx
@@ -126,25 +126,7 @@
     <t xml:space="preserve">10:00 - 11:00</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Cambria"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Rafael/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Cambria"/>
-        <family val="0"/>
-      </rPr>
-      <t xml:space="preserve">João Pedro</t>
-    </r>
+    <t xml:space="preserve">Rafael/João Pedro</t>
   </si>
   <si>
     <t xml:space="preserve">11:00 - 12:00</t>
@@ -153,25 +135,7 @@
     <t xml:space="preserve">Rafael (retornos dia 25)</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Cambria"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Gustavo/ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Cambria"/>
-        <family val="0"/>
-      </rPr>
-      <t xml:space="preserve">João Pedro</t>
-    </r>
+    <t xml:space="preserve">Gustavo/ João Pedro</t>
   </si>
   <si>
     <t xml:space="preserve">12:00 - 13:00</t>
@@ -192,25 +156,7 @@
     <t xml:space="preserve">14:00 - 15:00</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Cambria"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Rafael /</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Cambria"/>
-        <family val="0"/>
-      </rPr>
-      <t xml:space="preserve">João Pedro</t>
-    </r>
+    <t xml:space="preserve">Rafael /João Pedro</t>
   </si>
   <si>
     <t xml:space="preserve">15:00 - 16:00</t>
@@ -247,7 +193,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -292,12 +238,6 @@
       <name val="Cambria"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Cambria"/>
-      <family val="0"/>
     </font>
   </fonts>
   <fills count="7">
@@ -379,36 +319,40 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -725,891 +669,891 @@
   <dimension ref="B1:T41"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="7" min="3" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="25.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="26.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="26.68"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="22.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="22.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26.21"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="7" min="3" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="25.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="26.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="26.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="22.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="22.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="L2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="N2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="O2" s="2"/>
-      <c r="P2" s="2"/>
-      <c r="R2" s="3" t="s">
+      <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
+      <c r="R2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="S2" s="3"/>
-      <c r="T2" s="3"/>
+      <c r="S2" s="4"/>
+      <c r="T2" s="4"/>
     </row>
     <row r="3" customFormat="false" ht="39.55" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="5" t="s">
+      <c r="J3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="K3" s="5" t="s">
+      <c r="K3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="L3" s="5" t="s">
+      <c r="L3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="N3" s="5" t="s">
+      <c r="N3" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="O3" s="5"/>
-      <c r="P3" s="5"/>
-      <c r="R3" s="3" t="s">
+      <c r="O3" s="6"/>
+      <c r="P3" s="6"/>
+      <c r="R3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="S3" s="3" t="s">
+      <c r="S3" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="T3" s="3" t="s">
+      <c r="T3" s="4" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5" t="s">
+      <c r="F4" s="6"/>
+      <c r="G4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5" t="s">
+      <c r="I4" s="6"/>
+      <c r="J4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="K4" s="5" t="s">
+      <c r="K4" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="L4" s="5" t="s">
+      <c r="L4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="N4" s="5" t="s">
+      <c r="N4" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="O4" s="5"/>
-      <c r="P4" s="5"/>
-      <c r="R4" s="5" t="s">
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="R4" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="S4" s="5"/>
-      <c r="T4" s="5"/>
-    </row>
-    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="4" t="s">
+      <c r="S4" s="6"/>
+      <c r="T4" s="6"/>
+    </row>
+    <row r="5" customFormat="false" ht="26.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B5" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5" t="s">
+      <c r="D5" s="6"/>
+      <c r="E5" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5" t="s">
+      <c r="H5" s="6"/>
+      <c r="I5" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="J5" s="5" t="s">
+      <c r="J5" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="K5" s="5" t="s">
+      <c r="K5" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="L5" s="5" t="s">
+      <c r="L5" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="N5" s="5" t="s">
+      <c r="N5" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="O5" s="5"/>
-      <c r="P5" s="5"/>
-      <c r="R5" s="5" t="s">
+      <c r="O5" s="6"/>
+      <c r="P5" s="6"/>
+      <c r="R5" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="S5" s="5"/>
-      <c r="T5" s="5"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="4" t="s">
+      <c r="S5" s="6"/>
+      <c r="T5" s="6"/>
+    </row>
+    <row r="6" customFormat="false" ht="21.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="H6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="I6" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="J6" s="5" t="s">
+      <c r="J6" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="K6" s="5" t="s">
+      <c r="K6" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="L6" s="5" t="s">
+      <c r="L6" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="R6" s="5" t="s">
+      <c r="R6" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="S6" s="5"/>
-      <c r="T6" s="5"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="4" t="s">
+      <c r="S6" s="6"/>
+      <c r="T6" s="6"/>
+    </row>
+    <row r="7" customFormat="false" ht="21.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B7" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5" t="s">
+      <c r="F7" s="6"/>
+      <c r="G7" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="H7" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5" t="s">
+      <c r="I7" s="6"/>
+      <c r="J7" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="K7" s="5" t="s">
+      <c r="K7" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="L7" s="5" t="s">
+      <c r="L7" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="R7" s="5" t="s">
+      <c r="R7" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="S7" s="5"/>
-      <c r="T7" s="5"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G8" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="H8" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="I8" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="J8" s="5" t="s">
+      <c r="J8" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="K8" s="5" t="s">
+      <c r="K8" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="L8" s="5" t="s">
+      <c r="L8" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="R8" s="5" t="s">
+      <c r="R8" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="S8" s="5"/>
-      <c r="T8" s="5"/>
+      <c r="S8" s="6"/>
+      <c r="T8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5" t="s">
+      <c r="E9" s="6"/>
+      <c r="F9" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="G9" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="H9" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="I9" s="5" t="s">
+      <c r="I9" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="J9" s="5" t="s">
+      <c r="J9" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="K9" s="5" t="s">
+      <c r="K9" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="L9" s="5" t="s">
+      <c r="L9" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="R9" s="5" t="s">
+      <c r="R9" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="S9" s="5"/>
-      <c r="T9" s="5"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="4" t="s">
+      <c r="S9" s="6"/>
+      <c r="T9" s="6"/>
+    </row>
+    <row r="10" customFormat="false" ht="23.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5" t="s">
+      <c r="C10" s="6"/>
+      <c r="D10" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5" t="s">
+      <c r="G10" s="6"/>
+      <c r="H10" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="I10" s="5" t="s">
+      <c r="I10" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="R10" s="5" t="s">
+      <c r="J10" s="6"/>
+      <c r="K10" s="6"/>
+      <c r="L10" s="6"/>
+      <c r="R10" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="S10" s="5"/>
-      <c r="T10" s="5"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="4" t="s">
+      <c r="S10" s="6"/>
+      <c r="T10" s="6"/>
+    </row>
+    <row r="11" customFormat="false" ht="27.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B11" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5" t="s">
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5" t="s">
+      <c r="I11" s="6"/>
+      <c r="J11" s="6"/>
+      <c r="K11" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="L11" s="5"/>
-      <c r="R11" s="5" t="s">
+      <c r="L11" s="6"/>
+      <c r="R11" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="S11" s="5"/>
-      <c r="T11" s="5"/>
+      <c r="S11" s="6"/>
+      <c r="T11" s="6"/>
     </row>
     <row r="12" customFormat="false" ht="26.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="F12" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="G12" s="5" t="s">
+      <c r="G12" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H12" s="5" t="s">
+      <c r="H12" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="I12" s="5" t="s">
+      <c r="I12" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="J12" s="5" t="s">
+      <c r="J12" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="K12" s="5" t="s">
+      <c r="K12" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="L12" s="5" t="s">
+      <c r="L12" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="R12" s="5" t="s">
+      <c r="R12" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="S12" s="5"/>
-      <c r="T12" s="5"/>
+      <c r="S12" s="6"/>
+      <c r="T12" s="6"/>
     </row>
     <row r="13" customFormat="false" ht="26.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="F13" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="G13" s="5" t="s">
+      <c r="G13" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="H13" s="5" t="s">
+      <c r="H13" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="I13" s="5" t="s">
+      <c r="I13" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="J13" s="5" t="s">
+      <c r="J13" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="K13" s="5" t="s">
+      <c r="K13" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="L13" s="5" t="s">
+      <c r="L13" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="R13" s="5"/>
-      <c r="S13" s="5"/>
-      <c r="T13" s="5"/>
+      <c r="R13" s="6"/>
+      <c r="S13" s="6"/>
+      <c r="T13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="R14" s="4" t="n">
+      <c r="R14" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="S14" s="4" t="n">
+      <c r="S14" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="T14" s="4" t="n">
+      <c r="T14" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-      <c r="J15" s="1"/>
-      <c r="K15" s="1"/>
-      <c r="L15" s="1"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
+      <c r="L15" s="2"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-      <c r="J16" s="1"/>
-      <c r="K16" s="1"/>
-      <c r="L16" s="1"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
+      <c r="L16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
-      <c r="H17" s="7"/>
-      <c r="I17" s="7"/>
-      <c r="J17" s="7"/>
-      <c r="K17" s="7"/>
-      <c r="L17" s="7"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
+      <c r="K17" s="8"/>
+      <c r="L17" s="8"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7"/>
-      <c r="H18" s="7"/>
-      <c r="I18" s="7"/>
-      <c r="J18" s="7"/>
-      <c r="K18" s="7"/>
-      <c r="L18" s="7"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="8"/>
+      <c r="K18" s="8"/>
+      <c r="L18" s="8"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7"/>
-      <c r="G19" s="7"/>
-      <c r="H19" s="7"/>
-      <c r="I19" s="7"/>
-      <c r="J19" s="7"/>
-      <c r="K19" s="7"/>
-      <c r="L19" s="7"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
+      <c r="J19" s="8"/>
+      <c r="K19" s="8"/>
+      <c r="L19" s="8"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
-      <c r="G20" s="7"/>
-      <c r="H20" s="7"/>
-      <c r="I20" s="7"/>
-      <c r="J20" s="7"/>
-      <c r="K20" s="7"/>
-      <c r="L20" s="7"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="8"/>
+      <c r="J20" s="8"/>
+      <c r="K20" s="8"/>
+      <c r="L20" s="8"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="7"/>
-      <c r="H21" s="7"/>
-      <c r="I21" s="7"/>
-      <c r="J21" s="7"/>
-      <c r="K21" s="7"/>
-      <c r="L21" s="7"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="8"/>
+      <c r="J21" s="8"/>
+      <c r="K21" s="8"/>
+      <c r="L21" s="8"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
-      <c r="G22" s="7"/>
-      <c r="H22" s="7"/>
-      <c r="I22" s="7"/>
-      <c r="J22" s="7"/>
-      <c r="K22" s="7"/>
-      <c r="L22" s="7"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="8"/>
+      <c r="I22" s="8"/>
+      <c r="J22" s="8"/>
+      <c r="K22" s="8"/>
+      <c r="L22" s="8"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
-      <c r="G23" s="7"/>
-      <c r="H23" s="7"/>
-      <c r="I23" s="7"/>
-      <c r="J23" s="7"/>
-      <c r="K23" s="7"/>
-      <c r="L23" s="7"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="8"/>
+      <c r="J23" s="8"/>
+      <c r="K23" s="8"/>
+      <c r="L23" s="8"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C24" s="7"/>
-      <c r="D24" s="7"/>
-      <c r="E24" s="7"/>
-      <c r="F24" s="7"/>
-      <c r="G24" s="7"/>
-      <c r="H24" s="7"/>
-      <c r="I24" s="7"/>
-      <c r="J24" s="7"/>
-      <c r="K24" s="7"/>
-      <c r="L24" s="7"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+      <c r="G24" s="8"/>
+      <c r="H24" s="8"/>
+      <c r="I24" s="8"/>
+      <c r="J24" s="8"/>
+      <c r="K24" s="8"/>
+      <c r="L24" s="8"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="7"/>
-      <c r="F25" s="7"/>
-      <c r="G25" s="7"/>
-      <c r="H25" s="7"/>
-      <c r="I25" s="7"/>
-      <c r="J25" s="7"/>
-      <c r="K25" s="7"/>
-      <c r="L25" s="7"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="8"/>
+      <c r="I25" s="8"/>
+      <c r="J25" s="8"/>
+      <c r="K25" s="8"/>
+      <c r="L25" s="8"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="7"/>
-      <c r="F26" s="7"/>
-      <c r="G26" s="7"/>
-      <c r="H26" s="7"/>
-      <c r="I26" s="7"/>
-      <c r="J26" s="7"/>
-      <c r="K26" s="7"/>
-      <c r="L26" s="7"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
+      <c r="G26" s="8"/>
+      <c r="H26" s="8"/>
+      <c r="I26" s="8"/>
+      <c r="J26" s="8"/>
+      <c r="K26" s="8"/>
+      <c r="L26" s="8"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C27" s="7"/>
-      <c r="D27" s="7"/>
-      <c r="E27" s="7"/>
-      <c r="F27" s="7"/>
-      <c r="G27" s="7"/>
-      <c r="H27" s="7"/>
-      <c r="I27" s="7"/>
-      <c r="J27" s="7"/>
-      <c r="K27" s="7"/>
-      <c r="L27" s="7"/>
+      <c r="C27" s="8"/>
+      <c r="D27" s="8"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
+      <c r="G27" s="8"/>
+      <c r="H27" s="8"/>
+      <c r="I27" s="8"/>
+      <c r="J27" s="8"/>
+      <c r="K27" s="8"/>
+      <c r="L27" s="8"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="1" t="s">
+      <c r="B29" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
-      <c r="E29" s="1"/>
-      <c r="F29" s="1"/>
-      <c r="G29" s="1"/>
-      <c r="H29" s="1"/>
-      <c r="I29" s="1"/>
-      <c r="J29" s="1"/>
-      <c r="K29" s="1"/>
-      <c r="L29" s="1"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="2"/>
+      <c r="I29" s="2"/>
+      <c r="J29" s="2"/>
+      <c r="K29" s="2"/>
+      <c r="L29" s="2"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="1" t="s">
+      <c r="B30" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C30" s="1"/>
-      <c r="D30" s="1"/>
-      <c r="E30" s="1"/>
-      <c r="F30" s="1"/>
-      <c r="G30" s="1"/>
-      <c r="H30" s="1"/>
-      <c r="I30" s="1"/>
-      <c r="J30" s="1"/>
-      <c r="K30" s="1"/>
-      <c r="L30" s="1"/>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="2"/>
+      <c r="G30" s="2"/>
+      <c r="H30" s="2"/>
+      <c r="I30" s="2"/>
+      <c r="J30" s="2"/>
+      <c r="K30" s="2"/>
+      <c r="L30" s="2"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C31" s="7"/>
-      <c r="D31" s="7"/>
-      <c r="E31" s="7"/>
-      <c r="F31" s="7"/>
-      <c r="G31" s="7"/>
-      <c r="H31" s="7"/>
-      <c r="I31" s="7"/>
-      <c r="J31" s="7"/>
-      <c r="K31" s="7"/>
-      <c r="L31" s="7"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="8"/>
+      <c r="E31" s="8"/>
+      <c r="F31" s="8"/>
+      <c r="G31" s="8"/>
+      <c r="H31" s="8"/>
+      <c r="I31" s="8"/>
+      <c r="J31" s="8"/>
+      <c r="K31" s="8"/>
+      <c r="L31" s="8"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C32" s="7"/>
-      <c r="D32" s="7"/>
-      <c r="E32" s="7"/>
-      <c r="F32" s="7"/>
-      <c r="G32" s="7"/>
-      <c r="H32" s="7"/>
-      <c r="I32" s="7"/>
-      <c r="J32" s="7"/>
-      <c r="K32" s="7"/>
-      <c r="L32" s="7"/>
+      <c r="C32" s="8"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="8"/>
+      <c r="G32" s="8"/>
+      <c r="H32" s="8"/>
+      <c r="I32" s="8"/>
+      <c r="J32" s="8"/>
+      <c r="K32" s="8"/>
+      <c r="L32" s="8"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="6" t="s">
+      <c r="B33" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C33" s="7"/>
-      <c r="D33" s="7"/>
-      <c r="E33" s="7"/>
-      <c r="F33" s="7"/>
-      <c r="G33" s="7"/>
-      <c r="H33" s="7"/>
-      <c r="I33" s="7"/>
-      <c r="J33" s="7"/>
-      <c r="K33" s="7"/>
-      <c r="L33" s="7"/>
+      <c r="C33" s="8"/>
+      <c r="D33" s="8"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="8"/>
+      <c r="G33" s="8"/>
+      <c r="H33" s="8"/>
+      <c r="I33" s="8"/>
+      <c r="J33" s="8"/>
+      <c r="K33" s="8"/>
+      <c r="L33" s="8"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="6" t="s">
+      <c r="B34" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C34" s="7"/>
-      <c r="D34" s="7"/>
-      <c r="E34" s="7"/>
-      <c r="F34" s="7"/>
-      <c r="G34" s="7"/>
-      <c r="H34" s="7"/>
-      <c r="I34" s="7"/>
-      <c r="J34" s="7"/>
-      <c r="K34" s="7"/>
-      <c r="L34" s="7"/>
+      <c r="C34" s="8"/>
+      <c r="D34" s="8"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="8"/>
+      <c r="G34" s="8"/>
+      <c r="H34" s="8"/>
+      <c r="I34" s="8"/>
+      <c r="J34" s="8"/>
+      <c r="K34" s="8"/>
+      <c r="L34" s="8"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="6" t="s">
+      <c r="B35" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="C35" s="7"/>
-      <c r="D35" s="7"/>
-      <c r="E35" s="7"/>
-      <c r="F35" s="7"/>
-      <c r="G35" s="7"/>
-      <c r="H35" s="7"/>
-      <c r="I35" s="7"/>
-      <c r="J35" s="7"/>
-      <c r="K35" s="7"/>
-      <c r="L35" s="7"/>
+      <c r="C35" s="8"/>
+      <c r="D35" s="8"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="8"/>
+      <c r="G35" s="8"/>
+      <c r="H35" s="8"/>
+      <c r="I35" s="8"/>
+      <c r="J35" s="8"/>
+      <c r="K35" s="8"/>
+      <c r="L35" s="8"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="6" t="s">
+      <c r="B36" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="C36" s="7"/>
-      <c r="D36" s="7"/>
-      <c r="E36" s="7"/>
-      <c r="F36" s="7"/>
-      <c r="G36" s="7"/>
-      <c r="H36" s="7"/>
-      <c r="I36" s="7"/>
-      <c r="J36" s="7"/>
-      <c r="K36" s="7"/>
-      <c r="L36" s="7"/>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
+      <c r="G36" s="8"/>
+      <c r="H36" s="8"/>
+      <c r="I36" s="8"/>
+      <c r="J36" s="8"/>
+      <c r="K36" s="8"/>
+      <c r="L36" s="8"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="6" t="s">
+      <c r="B37" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C37" s="7"/>
-      <c r="D37" s="7"/>
-      <c r="E37" s="7"/>
-      <c r="F37" s="7"/>
-      <c r="G37" s="7"/>
-      <c r="H37" s="7"/>
-      <c r="I37" s="7"/>
-      <c r="J37" s="7"/>
-      <c r="K37" s="7"/>
-      <c r="L37" s="7"/>
+      <c r="C37" s="8"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="8"/>
+      <c r="F37" s="8"/>
+      <c r="G37" s="8"/>
+      <c r="H37" s="8"/>
+      <c r="I37" s="8"/>
+      <c r="J37" s="8"/>
+      <c r="K37" s="8"/>
+      <c r="L37" s="8"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="6" t="s">
+      <c r="B38" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C38" s="7"/>
-      <c r="D38" s="7"/>
-      <c r="E38" s="7"/>
-      <c r="F38" s="7"/>
-      <c r="G38" s="7"/>
-      <c r="H38" s="7"/>
-      <c r="I38" s="7"/>
-      <c r="J38" s="7"/>
-      <c r="K38" s="7"/>
-      <c r="L38" s="7"/>
+      <c r="C38" s="8"/>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="8"/>
+      <c r="G38" s="8"/>
+      <c r="H38" s="8"/>
+      <c r="I38" s="8"/>
+      <c r="J38" s="8"/>
+      <c r="K38" s="8"/>
+      <c r="L38" s="8"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="6" t="s">
+      <c r="B39" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="C39" s="7"/>
-      <c r="D39" s="7"/>
-      <c r="E39" s="7"/>
-      <c r="F39" s="7"/>
-      <c r="G39" s="7"/>
-      <c r="H39" s="7"/>
-      <c r="I39" s="7"/>
-      <c r="J39" s="7"/>
-      <c r="K39" s="7"/>
-      <c r="L39" s="7"/>
+      <c r="C39" s="8"/>
+      <c r="D39" s="8"/>
+      <c r="E39" s="8"/>
+      <c r="F39" s="8"/>
+      <c r="G39" s="8"/>
+      <c r="H39" s="8"/>
+      <c r="I39" s="8"/>
+      <c r="J39" s="8"/>
+      <c r="K39" s="8"/>
+      <c r="L39" s="8"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="6" t="s">
+      <c r="B40" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C40" s="7"/>
-      <c r="D40" s="7"/>
-      <c r="E40" s="7"/>
-      <c r="F40" s="7"/>
-      <c r="G40" s="7"/>
-      <c r="H40" s="7"/>
-      <c r="I40" s="7"/>
-      <c r="J40" s="7"/>
-      <c r="K40" s="7"/>
-      <c r="L40" s="7"/>
+      <c r="C40" s="8"/>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8"/>
+      <c r="F40" s="8"/>
+      <c r="G40" s="8"/>
+      <c r="H40" s="8"/>
+      <c r="I40" s="8"/>
+      <c r="J40" s="8"/>
+      <c r="K40" s="8"/>
+      <c r="L40" s="8"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="6" t="s">
+      <c r="B41" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C41" s="7"/>
-      <c r="D41" s="7"/>
-      <c r="E41" s="7"/>
-      <c r="F41" s="7"/>
-      <c r="G41" s="7"/>
-      <c r="H41" s="7"/>
-      <c r="I41" s="7"/>
-      <c r="J41" s="7"/>
-      <c r="K41" s="7"/>
-      <c r="L41" s="7"/>
+      <c r="C41" s="8"/>
+      <c r="D41" s="8"/>
+      <c r="E41" s="8"/>
+      <c r="F41" s="8"/>
+      <c r="G41" s="8"/>
+      <c r="H41" s="8"/>
+      <c r="I41" s="8"/>
+      <c r="J41" s="8"/>
+      <c r="K41" s="8"/>
+      <c r="L41" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>